<commit_message>
add flag to file to select GVFA only or Combined method
</commit_message>
<xml_diff>
--- a/Results/GVFA + Traditional feat results.xlsx
+++ b/Results/GVFA + Traditional feat results.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://latrobeuni-my.sharepoint.com/personal/22390013_students_ltu_edu_au/Documents/Projects/Molecular_Solubility/Molecular_solubility_traditional/Results/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="197" documentId="13_ncr:1_{D865690D-A916-4B50-AFA5-866BC8A56084}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{84CE4A10-58B2-4729-A437-A07A91616A06}"/>
+  <xr:revisionPtr revIDLastSave="215" documentId="13_ncr:1_{D865690D-A916-4B50-AFA5-866BC8A56084}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{81A66B79-33FE-4F3C-919E-3837A01C3553}"/>
   <bookViews>
-    <workbookView xWindow="15270" yWindow="-18240" windowWidth="29040" windowHeight="17520" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="2" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -18,6 +18,7 @@
     <sheet name="GVFA+edge" sheetId="3" r:id="rId3"/>
     <sheet name="Sheet2" sheetId="4" r:id="rId4"/>
     <sheet name="Teufel results" sheetId="5" r:id="rId5"/>
+    <sheet name="Sheet3" sheetId="6" r:id="rId6"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -40,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="316" uniqueCount="127">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="333" uniqueCount="144">
   <si>
     <t>Concatinate</t>
   </si>
@@ -466,6 +467,57 @@
   <si>
     <t>0.773 ± 0.02</t>
   </si>
+  <si>
+    <t>GVFA upodated code with edge feature, Not extended GVFA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0  XGB_298 concatinate GVFA(100)  0.41  0.3124  0.5589  0.9251  125 features + 128 fingerprint 7 f_group+38 </t>
+  </si>
+  <si>
+    <t>0  XGB_298 concatinate GVFA(200)  0.4137  0.3121  0.5587  0.9252  125 features + 128 fingerprint 7 f_group+38 fe...</t>
+  </si>
+  <si>
+    <t>0  XGB_298 concatinate GVFA(500)  0.412  0.3214  0.5669  0.9229  125 features + 128 fingerprint 7 f_group+38 fe...</t>
+  </si>
+  <si>
+    <t>0  XGB_298 concatinate GVFA(1000)  0.4202  0.33  0.5745  0.9209  125 features + 128 fingerprint 7 f_group+38 fe...</t>
+  </si>
+  <si>
+    <t>0  XGB_298 concatinate GVFA(2000)  0.4146  0.3235  0.5688  0.9224  125 features + 128 fingerprint 7 f_group+38 fe...</t>
+  </si>
+  <si>
+    <t>0  XGB_298 concatinate GVFA(5000)  0.4185  0.3333  0.5774  0.9201  125 features + 128 fingerprint 7 f_group+38 fe...</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OLD GVFA </t>
+  </si>
+  <si>
+    <t>0  XGB_298 concatinate GVFA(100)  0.4087  0.3127  0.5592  0.925  125 features + 128 fingerprint 7 f_group+38 fe...</t>
+  </si>
+  <si>
+    <t>0  XGB_298 concatinate GVFA(500)  0.4144  0.3311  0.5754  0.9206  125 features + 128 fingerprint 7 f_group+38 fe...</t>
+  </si>
+  <si>
+    <t>0  XGB_298 concatinate GVFA(1000)  0.4143  0.3282  0.5729  0.9213  125 features + 128 fingerprint 7 f_group+38 fe...</t>
+  </si>
+  <si>
+    <t>0  XGB_298 concatinate GVFA(2000)  0.4024  0.3116  0.5582  0.9253  125 features + 128 fingerprint 7 f_group+38 fe...</t>
+  </si>
+  <si>
+    <t>0  XGB_298 concatinate GVFA(5000)  0.4175  0.333  0.5771  0.9201  125 features + 128 fingerprint 7 f_group+38 fe...</t>
+  </si>
+  <si>
+    <t>Ridge      dim=10000 seed=0  MAE=0.7161  RMSE=0.9451  R2=0.7858  [mem] 2.00 GB</t>
+  </si>
+  <si>
+    <t>SVR        dim=10000 seed=0  MAE=0.7600  RMSE=0.9853  R2=0.7672  [mem] 3.20 GB</t>
+  </si>
+  <si>
+    <t>10_000</t>
+  </si>
+  <si>
+    <t>0  XGB_298 concatinate GVFA(10000)  0.4221  0.3461  0.5883  0.917  125 features + 128 fingerprint 7 f_group+38 fe...</t>
+  </si>
 </sst>
 </file>
 
@@ -474,7 +526,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0000"/>
   </numFmts>
-  <fonts count="15" x14ac:knownFonts="1">
+  <fonts count="16" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -572,8 +624,15 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF006100"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -596,6 +655,11 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFF2F2F2"/>
         <bgColor rgb="FFFFFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
       </patternFill>
     </fill>
   </fills>
@@ -623,10 +687,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="15" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -674,8 +739,10 @@
     <xf numFmtId="0" fontId="9" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="15" fillId="5" borderId="0" xfId="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Good" xfId="1" builtinId="26"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -689,6 +756,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2357,7 +2428,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B1816702-8316-4866-AF73-215B6F8716F8}">
-  <dimension ref="B1:AB104"/>
+  <dimension ref="B1:AB112"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="14" max="15" width="15" customWidth="1"/>
@@ -4438,34 +4509,58 @@
         <v>0.766 ± 0.01</v>
       </c>
     </row>
-    <row r="98" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="98" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B98" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="99" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="99" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B99" t="s">
         <v>101</v>
       </c>
     </row>
-    <row r="100" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="100" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B100" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="102" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="102" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B102" t="s">
         <v>103</v>
       </c>
     </row>
-    <row r="103" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="103" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B103" t="s">
         <v>104</v>
       </c>
     </row>
-    <row r="104" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="104" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B104" t="s">
         <v>105</v>
+      </c>
+    </row>
+    <row r="109" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B109" s="21" t="s">
+        <v>142</v>
+      </c>
+      <c r="C109" s="21"/>
+      <c r="D109" s="21"/>
+      <c r="E109" s="21"/>
+      <c r="F109" s="21"/>
+      <c r="G109" s="21"/>
+      <c r="H109" s="21"/>
+      <c r="I109" s="21"/>
+      <c r="J109" s="21"/>
+      <c r="K109" s="21"/>
+    </row>
+    <row r="111" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B111" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="112" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B112" t="s">
+        <v>141</v>
       </c>
     </row>
   </sheetData>
@@ -4478,4 +4573,84 @@
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A2B4BE4D-2707-4B2E-B264-E5074524D766}">
+  <dimension ref="A2:A18"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="8" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="9" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="12" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="13" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="14" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="15" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="16" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>143</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>